<commit_message>
feat: implement custom org chart layout with support for configurable node headcount and vertical/horizontal child distribution
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -406,6 +406,8 @@
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +432,12 @@
       <c r="G1" t="str">
         <v>badgeColor</v>
       </c>
+      <c r="H1" t="str">
+        <v>headcount</v>
+      </c>
+      <c r="I1" t="str">
+        <v>childLayout</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -453,6 +461,12 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="str">
+        <v>vertical</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -476,6 +490,12 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3" t="str">
+        <v>horizontal</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -499,6 +519,12 @@
       <c r="G4" t="str">
         <v/>
       </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="str">
+        <v>horizontal</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -522,6 +548,12 @@
       <c r="G5" t="str">
         <v/>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>horizontal</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -545,10 +577,16 @@
       <c r="G6" t="str">
         <v>#16A34A</v>
       </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="I6" t="str">
+        <v>horizontal</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>